<commit_message>
Data processing, modeling and comparison
</commit_message>
<xml_diff>
--- a/dashboard/model_comparison.xlsx
+++ b/dashboard/model_comparison.xlsx
@@ -459,7 +459,7 @@
         <v>14403.9</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3302500247955322</v>
+        <v>0.2996251583099365</v>
       </c>
     </row>
     <row r="3">
@@ -478,7 +478,7 @@
         <v>18886.9</v>
       </c>
       <c r="E3" t="n">
-        <v>8.275981187820435</v>
+        <v>9.380486011505127</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +497,7 @@
         <v>2896.8</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7017395496368408</v>
+        <v>0.8205738067626953</v>
       </c>
     </row>
     <row r="5">

</xml_diff>